<commit_message>
Dashboard HTML theo vai trò và trang Tóm tắt dạng dashboard trong Excel
- bao_cao.py + dashboard.html: dashboard tự chứa, chạy offline; xem theo
  vai trò Chủ shop / Quản lý / Kế toán, ý chính hôm nay, chỉ số, biểu đồ
  trạng thái và tiền về theo giờ, việc cần làm có nút chép tin nhắn,
  thu theo kênh, đơn lớn cần xem sao kê, hóa đơn điện tử, bảng đơn có lọc;
  sáng/tối, số đầy đủ/rút gọn, hiệu ứng, tối ưu desktop/tablet/điện thoại
- Excel: trang Tóm tắt thành dashboard (ô số liệu, biểu đồ, việc cần làm)
- agent.py: tùy chọn --doi-chieu-hoa-don, nhận cột Kênh bán, đọc giờ giao
  dịch trên ảnh dạng bảng
- Prompt chạy thử: đối chiếu hóa đơn trước rồi mở dashboard

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bo_du_lieu_mau_doi_soat/4-ket-qua-dung-san/1-doi-soat-chuyen-khoan.xlsx
+++ b/bo_du_lieu_mau_doi_soat/4-ket-qua-dung-san/1-doi-soat-chuyen-khoan.xlsx
@@ -21,8 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="4">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0&quot;đ&quot;"/>
+  </numFmts>
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,18 +33,61 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
-      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="18"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <color rgb="FF9CA3AF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
+      <color rgb="FF6B7280"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF1B1F24"/>
+      <sz val="24"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF6B7280"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF1B1F24"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF1B1F24"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF1B1F24"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF6B7280"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -71,11 +116,41 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF111827"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF9FAFB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE3F4E3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCEAE2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8E1E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3DB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -83,23 +158,140 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <top style="thick">
+        <color rgb="FF2A78D6"/>
+      </top>
+    </border>
+    <border>
+      <top style="thick">
+        <color rgb="FFD03B3B"/>
+      </top>
+    </border>
+    <border>
+      <top style="thick">
+        <color rgb="FF0CA30C"/>
+      </top>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="FFE5E7EB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -174,6 +366,268 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Giá trị đơn theo trạng thái</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tóm tắt'!D11</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <dPt>
+            <idx val="0"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="0CA30C"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="1"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="EC835A"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="2"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="D03B3B"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="3"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="FAB219"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <cat>
+            <numRef>
+              <f>'Tóm tắt'!$B$12:$B$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tóm tắt'!$D$12:$D$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="60"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Tiền về theo giờ (theo ảnh đã ghép)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tóm tắt'!C19</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2A78D6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tóm tắt'!$B$20:$B$26</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tóm tắt'!$C$20:$C$26</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="80"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4500000" cy="2232000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4500000" cy="2232000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -462,132 +916,613 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002A78D6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:M43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="110" customWidth="1" min="3" max="3"/>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="2" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="2" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="2" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Đối soát chuyển khoản · 12/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>16 đơn · 17 ảnh · phải thu 20.200.000đ · đã nhận theo ảnh 16.970.000đ</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+      <c r="M1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>ĐỐI SOÁT CHUYỂN KHOẢN · 12/10/2026</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>16 đơn · 17 ảnh · tạo lúc 20:59 12/10/2026</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+      <c r="M3" s="1" t="n"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>ĐÃ THU THEO ẢNH</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>CÒN PHẢI THU</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="n"/>
+      <c r="H5" s="7" t="n"/>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>ĐƠN SẴN SÀNG GIAO</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="n"/>
+      <c r="L5" s="9" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="B6" s="10" t="n">
+        <v>16970000</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>3250000</v>
+      </c>
+      <c r="J6" s="11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1"/>
+    <row r="8">
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>84% của 20.200.000đ phải thu</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="n"/>
+      <c r="D8" s="13" t="n"/>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>6 đơn chưa xong</t>
+        </is>
+      </c>
+      <c r="G8" s="13" t="n"/>
+      <c r="H8" s="13" t="n"/>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>trên 16 đơn</t>
+        </is>
+      </c>
+      <c r="K8" s="13" t="n"/>
+      <c r="L8" s="13" t="n"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>THEO TRẠNG THÁI</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>Trạng thái</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>Số đơn</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Đơn</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Giá trị đơn</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Đã nhận</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Còn thiếu</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>Đã trả đủ</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="C12" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>DH1001 Nguyễn Văn An; DH1003 Lê Minh Châu; DH1005 Hoàng Thu Hà; DH1007 Đỗ Gia Huy; DH1008 Công ty TNHH Nội thất Gỗ Việt; DH1010 Đặng Hữu Phước; DH1012 Công ty CP Sự kiện Ánh Dương; DH1013 Trịnh Văn Long; DH1014 Trịnh Văn Long; DH1015 Lý Thanh Tâm</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="D12" s="19" t="n">
+        <v>15470000</v>
+      </c>
+      <c r="F12" s="19" t="n">
+        <v>15470000</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>Trả thiếu</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="C13" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>DH1002 Trần Thị Bình (thiếu 500.000đ)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="D13" s="19" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="F13" s="19" t="n">
+        <v>700000</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="21" t="inlineStr">
         <is>
           <t>Chưa trả</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="C14" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>DH1004 Phạm Quốc Dũng (890.000đ); DH1016 Mai Phương Thảo (990.000đ)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="D14" s="19" t="n">
+        <v>1880000</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>1880000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="22" t="inlineStr">
         <is>
           <t>Cần kiểm tra</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="C15" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>DH1006 Võ Thanh Em; DH1009 Bùi Ngọc Lan; DH1011 Ngô Thị Kim</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Ảnh</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>17</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Đã ghép 12 · Trùng 1 · Cần xem 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Lưu ý: số tiền lấy từ ảnh khách gửi. Đơn giá trị lớn cần xem sao kê ngân hàng trước khi giao. Agent không gửi tin nhắn; cột tin nhắn chỉ là bản soạn sẵn.</t>
+      <c r="D15" s="19" t="n">
+        <v>1650000</v>
+      </c>
+      <c r="F15" s="19" t="n">
+        <v>800000</v>
+      </c>
+      <c r="G15" s="19" t="n">
+        <v>870000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>TIỀN VỀ THEO GIỜ</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>Giờ</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Số tiền</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Giao dịch</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="n">
+        <v>450000</v>
+      </c>
+      <c r="D20" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="23" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="n">
+        <v>1020000</v>
+      </c>
+      <c r="D21" s="18" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="23" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="n">
+        <v>300000</v>
+      </c>
+      <c r="D22" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="n">
+        <v>7700000</v>
+      </c>
+      <c r="D23" s="18" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="23" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="n">
+        <v>350000</v>
+      </c>
+      <c r="D24" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="23" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="n">
+        <v>4790000</v>
+      </c>
+      <c r="D25" s="18" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="23" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C26" s="19" t="n">
+        <v>2360000</v>
+      </c>
+      <c r="D26" s="18" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>VIỆC CẦN LÀM</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="15" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+      <c r="C33" s="15" t="inlineStr">
+        <is>
+          <t>Mã đơn</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="inlineStr">
+        <is>
+          <t>Khách hàng</t>
+        </is>
+      </c>
+      <c r="F33" s="15" t="inlineStr">
+        <is>
+          <t>SĐT</t>
+        </is>
+      </c>
+      <c r="G33" s="16" t="inlineStr">
+        <is>
+          <t>Còn thiếu</t>
+        </is>
+      </c>
+      <c r="H33" s="15" t="inlineStr">
+        <is>
+          <t>Việc cần làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="20" t="inlineStr">
+        <is>
+          <t>Trả thiếu</t>
+        </is>
+      </c>
+      <c r="C34" s="23" t="inlineStr">
+        <is>
+          <t>DH1002</t>
+        </is>
+      </c>
+      <c r="D34" s="23" t="inlineStr">
+        <is>
+          <t>Trần Thị Bình</t>
+        </is>
+      </c>
+      <c r="F34" s="23" t="inlineStr">
+        <is>
+          <t>0902222333</t>
+        </is>
+      </c>
+      <c r="G34" s="19" t="n">
+        <v>500000</v>
+      </c>
+      <c r="H34" s="24" t="inlineStr">
+        <is>
+          <t>Nhắc khách chuyển thêm 500.000đ</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="21" t="inlineStr">
+        <is>
+          <t>Chưa trả</t>
+        </is>
+      </c>
+      <c r="C35" s="23" t="inlineStr">
+        <is>
+          <t>DH1004</t>
+        </is>
+      </c>
+      <c r="D35" s="23" t="inlineStr">
+        <is>
+          <t>Phạm Quốc Dũng</t>
+        </is>
+      </c>
+      <c r="F35" s="23" t="inlineStr">
+        <is>
+          <t>0904444555</t>
+        </is>
+      </c>
+      <c r="G35" s="19" t="n">
+        <v>890000</v>
+      </c>
+      <c r="H35" s="24" t="inlineStr">
+        <is>
+          <t>Chưa tìm thấy ảnh ghép chắc; kiểm tra Zalo/sao kê trước khi nhắc khách</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="21" t="inlineStr">
+        <is>
+          <t>Chưa trả</t>
+        </is>
+      </c>
+      <c r="C36" s="23" t="inlineStr">
+        <is>
+          <t>DH1016</t>
+        </is>
+      </c>
+      <c r="D36" s="23" t="inlineStr">
+        <is>
+          <t>Mai Phương Thảo</t>
+        </is>
+      </c>
+      <c r="F36" s="23" t="inlineStr">
+        <is>
+          <t>0918000111</t>
+        </is>
+      </c>
+      <c r="G36" s="19" t="n">
+        <v>990000</v>
+      </c>
+      <c r="H36" s="24" t="inlineStr">
+        <is>
+          <t>Chưa tìm thấy ảnh ghép chắc; kiểm tra Zalo/sao kê trước khi nhắc khách</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="22" t="inlineStr">
+        <is>
+          <t>Cần kiểm tra</t>
+        </is>
+      </c>
+      <c r="C37" s="23" t="inlineStr">
+        <is>
+          <t>DH1006</t>
+        </is>
+      </c>
+      <c r="D37" s="23" t="inlineStr">
+        <is>
+          <t>Võ Thanh Em</t>
+        </is>
+      </c>
+      <c r="F37" s="23" t="inlineStr">
+        <is>
+          <t>0906666777</t>
+        </is>
+      </c>
+      <c r="G37" s="19" t="n">
+        <v>250000</v>
+      </c>
+      <c r="H37" s="24" t="inlineStr">
+        <is>
+          <t>Mở ảnh z6042817840331_e0d5b8.jpg (chỉ đúng số tiền, chưa đủ để ghép) để xác nhận</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="22" t="inlineStr">
+        <is>
+          <t>Cần kiểm tra</t>
+        </is>
+      </c>
+      <c r="C38" s="23" t="inlineStr">
+        <is>
+          <t>DH1009</t>
+        </is>
+      </c>
+      <c r="D38" s="23" t="inlineStr">
+        <is>
+          <t>Bùi Ngọc Lan</t>
+        </is>
+      </c>
+      <c r="F38" s="23" t="inlineStr">
+        <is>
+          <t>0909999000</t>
+        </is>
+      </c>
+      <c r="G38" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="24" t="inlineStr">
+        <is>
+          <t>Nhận dư 20.000đ; xác minh hoàn tiền hoặc trừ đơn sau</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="22" t="inlineStr">
+        <is>
+          <t>Cần kiểm tra</t>
+        </is>
+      </c>
+      <c r="C39" s="23" t="inlineStr">
+        <is>
+          <t>DH1011</t>
+        </is>
+      </c>
+      <c r="D39" s="23" t="inlineStr">
+        <is>
+          <t>Ngô Thị Kim</t>
+        </is>
+      </c>
+      <c r="F39" s="23" t="inlineStr">
+        <is>
+          <t>0913444555</t>
+        </is>
+      </c>
+      <c r="G39" s="19" t="n">
+        <v>620000</v>
+      </c>
+      <c r="H39" s="24" t="inlineStr">
+        <is>
+          <t>Mở ảnh z6042818350288_6ac2e5.jpg (có mã đơn nhưng không đọc được số tiền) để xác nhận</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="25" t="inlineStr">
+        <is>
+          <t>Ảnh: 17 · ghép tự động 12 (75%) · trùng 1 · cần xem 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="25" t="inlineStr">
+        <is>
+          <t>Hóa đơn điện tử: 8 số · khớp 2 · lệch 3 · tải trùng 1 · chỉ có ở một bên 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="25" t="inlineStr">
+        <is>
+          <t>Số tiền lấy từ ảnh khách gửi, chưa phải xác nhận tiền đã vào tài khoản. Xem sao kê trước khi giao đơn lớn. Agent không gửi tin nhắn.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="J6:L7"/>
+    <mergeCell ref="B6:D7"/>
+    <mergeCell ref="F6:H7"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -614,791 +1549,791 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>Mã đơn</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="26" t="inlineStr">
         <is>
           <t>Khách hàng</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="26" t="inlineStr">
         <is>
           <t>Số điện thoại</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="26" t="inlineStr">
         <is>
           <t>Phải thu</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="26" t="inlineStr">
         <is>
           <t>Đã nhận theo ảnh</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="26" t="inlineStr">
         <is>
           <t>Còn thiếu</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="26" t="inlineStr">
         <is>
           <t>Trạng thái</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" s="26" t="inlineStr">
         <is>
           <t>Ảnh đã ghép</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I1" s="26" t="inlineStr">
         <is>
           <t>Căn cứ ghép</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="J1" s="26" t="inlineStr">
         <is>
           <t>Việc cần làm</t>
         </is>
       </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="K1" s="26" t="inlineStr">
         <is>
           <t>Tin nhắn nhắc (soạn sẵn, chưa gửi)</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="27" t="inlineStr">
         <is>
           <t>DH1001</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="27" t="inlineStr">
         <is>
           <t>Nguyễn Văn An</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="27" t="inlineStr">
         <is>
           <t>0901111222</t>
         </is>
       </c>
-      <c r="D2" s="8" t="n">
+      <c r="D2" s="28" t="n">
         <v>450000</v>
       </c>
-      <c r="E2" s="8" t="n">
+      <c r="E2" s="28" t="n">
         <v>450000</v>
       </c>
-      <c r="F2" s="8" t="n">
+      <c r="F2" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="27" t="inlineStr">
         <is>
           <t>Đã trả đủ</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="29" t="inlineStr">
         <is>
           <t>z6042817353390_8f1c2a.jpg</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" s="29" t="inlineStr">
         <is>
           <t>có mã đơn, có tên khách, đúng số tiền</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>Xác nhận đơn</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="J2" s="29" t="inlineStr">
+        <is>
+          <t>Đủ theo ảnh; kiểm tra sao kê theo quy trình trước khi xác nhận đơn</t>
+        </is>
+      </c>
+      <c r="K2" s="29" t="inlineStr"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="30" t="inlineStr">
         <is>
           <t>DH1002</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="30" t="inlineStr">
         <is>
           <t>Trần Thị Bình</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="30" t="inlineStr">
         <is>
           <t>0902222333</t>
         </is>
       </c>
-      <c r="D3" s="9" t="n">
+      <c r="D3" s="31" t="n">
         <v>1200000</v>
       </c>
-      <c r="E3" s="9" t="n">
+      <c r="E3" s="31" t="n">
         <v>700000</v>
       </c>
-      <c r="F3" s="9" t="n">
+      <c r="F3" s="31" t="n">
         <v>500000</v>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="30" t="inlineStr">
         <is>
           <t>Trả thiếu</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="32" t="inlineStr">
         <is>
           <t>z6042817411205_a7d3e9.jpg</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="32" t="inlineStr">
         <is>
           <t>có mã đơn</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="32" t="inlineStr">
         <is>
           <t>Nhắc khách chuyển thêm 500.000đ</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="K3" s="32" t="inlineStr">
         <is>
           <t>Chào Trần Thị Bình, shop đã nhận 700.000đ cho đơn DH1002. Đơn còn thiếu 500.000đ, anh/chị kiểm tra giúp shop nhé. Cảm ơn anh/chị!</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="27" t="inlineStr">
         <is>
           <t>DH1003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="27" t="inlineStr">
         <is>
           <t>Lê Minh Châu</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="27" t="inlineStr">
         <is>
           <t>0912345678</t>
         </is>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="28" t="n">
         <v>320000</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="28" t="n">
         <v>320000</v>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="F4" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="27" t="inlineStr">
         <is>
           <t>Đã trả đủ</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="29" t="inlineStr">
         <is>
           <t>z6042817502117_3b9e01.jpg</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="29" t="inlineStr">
         <is>
           <t>có số điện thoại, đúng số tiền</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Xác nhận đơn</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="J4" s="29" t="inlineStr">
+        <is>
+          <t>Đủ theo ảnh; kiểm tra sao kê theo quy trình trước khi xác nhận đơn</t>
+        </is>
+      </c>
+      <c r="K4" s="29" t="inlineStr"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="33" t="inlineStr">
         <is>
           <t>DH1004</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="33" t="inlineStr">
         <is>
           <t>Phạm Quốc Dũng</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="33" t="inlineStr">
         <is>
           <t>0904444555</t>
         </is>
       </c>
-      <c r="D5" s="10" t="n">
+      <c r="D5" s="34" t="n">
         <v>890000</v>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="E5" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="10" t="n">
+      <c r="F5" s="34" t="n">
         <v>890000</v>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="33" t="inlineStr">
         <is>
           <t>Chưa trả</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr"/>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>Nhắc khách thanh toán</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>Chào Phạm Quốc Dũng, đơn DH1004 (890.000đ) shop chưa thấy thanh toán. Nếu anh/chị đã chuyển, gửi giúp shop ảnh chuyển khoản nhé. Cảm ơn anh/chị!</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="H5" s="35" t="inlineStr"/>
+      <c r="I5" s="35" t="inlineStr"/>
+      <c r="J5" s="35" t="inlineStr">
+        <is>
+          <t>Chưa tìm thấy ảnh ghép chắc; kiểm tra Zalo/sao kê trước khi nhắc khách</t>
+        </is>
+      </c>
+      <c r="K5" s="35" t="inlineStr">
+        <is>
+          <t>Chào Phạm Quốc Dũng, với đơn DH1004 (890.000đ), shop chưa ghép được ảnh thanh toán trong dữ liệu cuối ngày. Nếu anh/chị đã chuyển, gửi giúp shop ảnh chuyển khoản nhé. Cảm ơn anh/chị!</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="27" t="inlineStr">
         <is>
           <t>DH1005</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="27" t="inlineStr">
         <is>
           <t>Hoàng Thu Hà</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="27" t="inlineStr">
         <is>
           <t>0905555666</t>
         </is>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="28" t="n">
         <v>560000</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="28" t="n">
         <v>560000</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="27" t="inlineStr">
         <is>
           <t>Đã trả đủ</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="29" t="inlineStr">
         <is>
           <t>z6042817618842_c41f77.jpg, z6042817733015_77ab02.jpg</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="29" t="inlineStr">
         <is>
           <t>có mã đơn, có tên khách</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>Xác nhận đơn</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="J6" s="29" t="inlineStr">
+        <is>
+          <t>Đủ theo ảnh; kiểm tra sao kê theo quy trình trước khi xác nhận đơn</t>
+        </is>
+      </c>
+      <c r="K6" s="29" t="inlineStr"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="36" t="inlineStr">
         <is>
           <t>DH1006</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="36" t="inlineStr">
         <is>
           <t>Võ Thanh Em</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="36" t="inlineStr">
         <is>
           <t>0906666777</t>
         </is>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="37" t="n">
         <v>250000</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="F7" s="11" t="n">
+      <c r="F7" s="37" t="n">
         <v>250000</v>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="36" t="inlineStr">
         <is>
           <t>Cần kiểm tra</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr"/>
-      <c r="I7" s="6" t="inlineStr"/>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="H7" s="38" t="inlineStr"/>
+      <c r="I7" s="38" t="inlineStr"/>
+      <c r="J7" s="38" t="inlineStr">
         <is>
           <t>Mở ảnh z6042817840331_e0d5b8.jpg (chỉ đúng số tiền, chưa đủ để ghép) để xác nhận</t>
         </is>
       </c>
-      <c r="K7" s="6" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="K7" s="38" t="inlineStr"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="27" t="inlineStr">
         <is>
           <t>DH1007</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="27" t="inlineStr">
         <is>
           <t>Đỗ Gia Huy</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="27" t="inlineStr">
         <is>
           <t>0907777888</t>
         </is>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="28" t="n">
         <v>1500000</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="28" t="n">
         <v>1500000</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="27" t="inlineStr">
         <is>
           <t>Đã trả đủ</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" s="29" t="inlineStr">
         <is>
           <t>z6042817921456_19ce4d.jpg</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I8" s="29" t="inlineStr">
         <is>
           <t>có tên khách, đúng số tiền</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>Xác nhận đơn</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="J8" s="29" t="inlineStr">
+        <is>
+          <t>Đủ theo ảnh; kiểm tra sao kê theo quy trình trước khi xác nhận đơn</t>
+        </is>
+      </c>
+      <c r="K8" s="29" t="inlineStr"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="27" t="inlineStr">
         <is>
           <t>DH1008</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="27" t="inlineStr">
         <is>
           <t>Công ty TNHH Nội thất Gỗ Việt</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="27" t="inlineStr">
         <is>
           <t>0243888999</t>
         </is>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="28" t="n">
         <v>5400000</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="28" t="n">
         <v>5400000</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="27" t="inlineStr">
         <is>
           <t>Đã trả đủ</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H9" s="29" t="inlineStr">
         <is>
           <t>z6042818034470_5d2a90.png</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I9" s="29" t="inlineStr">
         <is>
           <t>có mã đơn, có tên khách, đúng số tiền</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t>Đủ theo ảnh; đơn lớn, xem sao kê trước khi giao</t>
-        </is>
-      </c>
-      <c r="K9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="J9" s="29" t="inlineStr">
+        <is>
+          <t>Đủ theo ảnh; xem sao kê trước khi xác nhận đơn hoặc giao hàng</t>
+        </is>
+      </c>
+      <c r="K9" s="29" t="inlineStr"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="36" t="inlineStr">
         <is>
           <t>DH1009</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="36" t="inlineStr">
         <is>
           <t>Bùi Ngọc Lan</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="36" t="inlineStr">
         <is>
           <t>0909999000</t>
         </is>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="37" t="n">
         <v>780000</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="37" t="n">
         <v>800000</v>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G10" s="36" t="inlineStr">
         <is>
           <t>Cần kiểm tra</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H10" s="38" t="inlineStr">
         <is>
           <t>z6042818115902_b8e6c3.jpg</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="I10" s="38" t="inlineStr">
         <is>
           <t>có mã đơn, có tên khách</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="J10" s="38" t="inlineStr">
         <is>
           <t>Nhận dư 20.000đ; xác minh hoàn tiền hoặc trừ đơn sau</t>
         </is>
       </c>
-      <c r="K10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="K10" s="38" t="inlineStr"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t>DH1010</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="27" t="inlineStr">
         <is>
           <t>Đặng Hữu Phước</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="27" t="inlineStr">
         <is>
           <t>0911222333</t>
         </is>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="28" t="n">
         <v>350000</v>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="28" t="n">
         <v>350000</v>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F11" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" s="27" t="inlineStr">
         <is>
           <t>Đã trả đủ</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H11" s="29" t="inlineStr">
         <is>
           <t>z6042818207719_0f4ad1.jpg</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="I11" s="29" t="inlineStr">
         <is>
           <t>có mã đơn, có tên khách, đúng số tiền</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>Xác nhận đơn</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="J11" s="29" t="inlineStr">
+        <is>
+          <t>Đủ theo ảnh; kiểm tra sao kê theo quy trình trước khi xác nhận đơn</t>
+        </is>
+      </c>
+      <c r="K11" s="29" t="inlineStr"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="36" t="inlineStr">
         <is>
           <t>DH1011</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="36" t="inlineStr">
         <is>
           <t>Ngô Thị Kim</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="36" t="inlineStr">
         <is>
           <t>0913444555</t>
         </is>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D12" s="37" t="n">
         <v>620000</v>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="F12" s="37" t="n">
         <v>620000</v>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G12" s="36" t="inlineStr">
         <is>
           <t>Cần kiểm tra</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr"/>
-      <c r="I12" s="6" t="inlineStr"/>
-      <c r="J12" s="6" t="inlineStr">
+      <c r="H12" s="38" t="inlineStr"/>
+      <c r="I12" s="38" t="inlineStr"/>
+      <c r="J12" s="38" t="inlineStr">
         <is>
           <t>Mở ảnh z6042818350288_6ac2e5.jpg (có mã đơn nhưng không đọc được số tiền) để xác nhận</t>
         </is>
       </c>
-      <c r="K12" s="6" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="K12" s="38" t="inlineStr"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>DH1012</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="27" t="inlineStr">
         <is>
           <t>Công ty CP Sự kiện Ánh Dương</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="27" t="inlineStr">
         <is>
           <t>0283777666</t>
         </is>
       </c>
-      <c r="D13" s="8" t="n">
+      <c r="D13" s="28" t="n">
         <v>3240000</v>
       </c>
-      <c r="E13" s="8" t="n">
+      <c r="E13" s="28" t="n">
         <v>3240000</v>
       </c>
-      <c r="F13" s="8" t="n">
+      <c r="F13" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G13" s="27" t="inlineStr">
         <is>
           <t>Đã trả đủ</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H13" s="29" t="inlineStr">
         <is>
           <t>z6042818462531_2e7b9f.png</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="I13" s="29" t="inlineStr">
         <is>
           <t>có mã đơn, có tên khách, đúng số tiền</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>Đủ theo ảnh; đơn lớn, xem sao kê trước khi giao</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="J13" s="29" t="inlineStr">
+        <is>
+          <t>Đủ theo ảnh; xem sao kê trước khi xác nhận đơn hoặc giao hàng</t>
+        </is>
+      </c>
+      <c r="K13" s="29" t="inlineStr"/>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="27" t="inlineStr">
         <is>
           <t>DH1013</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="27" t="inlineStr">
         <is>
           <t>Trịnh Văn Long</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="27" t="inlineStr">
         <is>
           <t>0915666777</t>
         </is>
       </c>
-      <c r="D14" s="8" t="n">
+      <c r="D14" s="28" t="n">
         <v>1150000</v>
       </c>
-      <c r="E14" s="8" t="n">
+      <c r="E14" s="28" t="n">
         <v>1150000</v>
       </c>
-      <c r="F14" s="8" t="n">
+      <c r="F14" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G14" s="27" t="inlineStr">
         <is>
           <t>Đã trả đủ</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H14" s="29" t="inlineStr">
         <is>
           <t>z6042818573004_d9f310.jpg</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="I14" s="29" t="inlineStr">
         <is>
           <t>1 lần chuyển cho 2 đơn: có mã các đơn, tổng tiền khớp</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>Xác nhận đơn</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="J14" s="29" t="inlineStr">
+        <is>
+          <t>Đủ theo ảnh; kiểm tra sao kê theo quy trình trước khi xác nhận đơn</t>
+        </is>
+      </c>
+      <c r="K14" s="29" t="inlineStr"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="27" t="inlineStr">
         <is>
           <t>DH1014</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="27" t="inlineStr">
         <is>
           <t>Trịnh Văn Long</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="27" t="inlineStr">
         <is>
           <t>0915666777</t>
         </is>
       </c>
-      <c r="D15" s="8" t="n">
+      <c r="D15" s="28" t="n">
         <v>400000</v>
       </c>
-      <c r="E15" s="8" t="n">
+      <c r="E15" s="28" t="n">
         <v>400000</v>
       </c>
-      <c r="F15" s="8" t="n">
+      <c r="F15" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G15" s="27" t="inlineStr">
         <is>
           <t>Đã trả đủ</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H15" s="29" t="inlineStr">
         <is>
           <t>z6042818573004_d9f310.jpg</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="I15" s="29" t="inlineStr">
         <is>
           <t>1 lần chuyển cho 2 đơn: có mã các đơn, tổng tiền khớp</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>Xác nhận đơn</t>
-        </is>
-      </c>
-      <c r="K15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="J15" s="29" t="inlineStr">
+        <is>
+          <t>Đủ theo ảnh; kiểm tra sao kê theo quy trình trước khi xác nhận đơn</t>
+        </is>
+      </c>
+      <c r="K15" s="29" t="inlineStr"/>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="27" t="inlineStr">
         <is>
           <t>DH1015</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="27" t="inlineStr">
         <is>
           <t>Lý Thanh Tâm</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="27" t="inlineStr">
         <is>
           <t>0917888999</t>
         </is>
       </c>
-      <c r="D16" s="8" t="n">
+      <c r="D16" s="28" t="n">
         <v>2100000</v>
       </c>
-      <c r="E16" s="8" t="n">
+      <c r="E16" s="28" t="n">
         <v>2100000</v>
       </c>
-      <c r="F16" s="8" t="n">
+      <c r="F16" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G16" s="27" t="inlineStr">
         <is>
           <t>Đã trả đủ</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="H16" s="29" t="inlineStr">
         <is>
           <t>z6042818680147_41b8ac.jpg</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="I16" s="29" t="inlineStr">
         <is>
           <t>có mã đơn, có tên khách, đúng số tiền</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t>Đủ theo ảnh; đơn lớn, xem sao kê trước khi giao</t>
-        </is>
-      </c>
-      <c r="K16" s="3" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="J16" s="29" t="inlineStr">
+        <is>
+          <t>Đủ theo ảnh; xem sao kê trước khi xác nhận đơn hoặc giao hàng</t>
+        </is>
+      </c>
+      <c r="K16" s="29" t="inlineStr"/>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="33" t="inlineStr">
         <is>
           <t>DH1016</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="33" t="inlineStr">
         <is>
           <t>Mai Phương Thảo</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="33" t="inlineStr">
         <is>
           <t>0918000111</t>
         </is>
       </c>
-      <c r="D17" s="10" t="n">
+      <c r="D17" s="34" t="n">
         <v>990000</v>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="E17" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="F17" s="10" t="n">
+      <c r="F17" s="34" t="n">
         <v>990000</v>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" s="33" t="inlineStr">
         <is>
           <t>Chưa trả</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr"/>
-      <c r="I17" s="5" t="inlineStr"/>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>Nhắc khách thanh toán</t>
-        </is>
-      </c>
-      <c r="K17" s="5" t="inlineStr">
-        <is>
-          <t>Chào Mai Phương Thảo, đơn DH1016 (990.000đ) shop chưa thấy thanh toán. Nếu anh/chị đã chuyển, gửi giúp shop ảnh chuyển khoản nhé. Cảm ơn anh/chị!</t>
+      <c r="H17" s="35" t="inlineStr"/>
+      <c r="I17" s="35" t="inlineStr"/>
+      <c r="J17" s="35" t="inlineStr">
+        <is>
+          <t>Chưa tìm thấy ảnh ghép chắc; kiểm tra Zalo/sao kê trước khi nhắc khách</t>
+        </is>
+      </c>
+      <c r="K17" s="35" t="inlineStr">
+        <is>
+          <t>Chào Mai Phương Thảo, với đơn DH1016 (990.000đ), shop chưa ghép được ảnh thanh toán trong dữ liệu cuối ngày. Nếu anh/chị đã chuyển, gửi giúp shop ảnh chuyển khoản nhé. Cảm ơn anh/chị!</t>
         </is>
       </c>
     </row>
@@ -1430,102 +2365,102 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>Tệp ảnh</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="26" t="inlineStr">
         <is>
           <t>Số tiền đọc được</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="26" t="inlineStr">
         <is>
           <t>Nội dung</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="26" t="inlineStr">
         <is>
           <t>Người chuyển</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="26" t="inlineStr">
         <is>
           <t>Mã giao dịch</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="26" t="inlineStr">
         <is>
           <t>Thời gian</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="26" t="inlineStr">
         <is>
           <t>Ghép vào đơn</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" s="26" t="inlineStr">
         <is>
           <t>Căn cứ</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I1" s="26" t="inlineStr">
         <is>
           <t>Kết quả</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="J1" s="26" t="inlineStr">
         <is>
           <t>Chữ đọc được trên ảnh</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="39" t="inlineStr">
         <is>
           <t>z6042817353390_8f1c2a.jpg</t>
         </is>
       </c>
-      <c r="B2" s="8" t="n">
+      <c r="B2" s="40" t="n">
         <v>450000</v>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="39" t="inlineStr">
         <is>
           <t>DH1001 NGUYEN VAN AN</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="39" t="inlineStr">
         <is>
           <t>NGUYEN VAN AN</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="39" t="inlineStr">
         <is>
           <t>FT26285104411</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="39" t="inlineStr">
         <is>
           <t>12/10/2026 08:41:07</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="39" t="inlineStr">
         <is>
           <t>DH1001</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="39" t="inlineStr">
         <is>
           <t>có mã đơn, có tên khách, đúng số tiền</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" s="39" t="inlineStr">
         <is>
           <t>Đã ghép</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J2" s="39" t="inlineStr">
         <is>
           <t>08:41 al RKM
 Sen Vàng Bank
@@ -1542,46 +2477,46 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="39" t="inlineStr">
         <is>
           <t>z6042817411205_a7d3e9.jpg</t>
         </is>
       </c>
-      <c r="B3" s="8" t="n">
+      <c r="B3" s="40" t="n">
         <v>700000</v>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="39" t="inlineStr">
         <is>
           <t>DH1002 chuyen truoc</t>
         </is>
       </c>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="D3" s="39" t="n"/>
+      <c r="E3" s="39" t="inlineStr">
         <is>
           <t>FT26285219034</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="39" t="inlineStr">
         <is>
           <t>12/10/2026 09:12:45</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="39" t="inlineStr">
         <is>
           <t>DH1002</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="39" t="inlineStr">
         <is>
           <t>có mã đơn</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I3" s="39" t="inlineStr">
         <is>
           <t>Đã ghép</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J3" s="39" t="inlineStr">
         <is>
           <t>09:12 | o_o
 Bién Xanh Bank
@@ -1599,46 +2534,46 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="39" t="inlineStr">
         <is>
           <t>z6042817502117_3b9e01.jpg</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="40" t="n">
         <v>320000</v>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="39" t="inlineStr">
         <is>
           <t>0912345678 thanh toan</t>
         </is>
       </c>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="D4" s="39" t="n"/>
+      <c r="E4" s="39" t="inlineStr">
         <is>
           <t>MM2610120933</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="39" t="inlineStr">
         <is>
           <t>09:33 - 12/10/2026</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="39" t="inlineStr">
         <is>
           <t>DH1003</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="39" t="inlineStr">
         <is>
           <t>có số điện thoại, đúng số tiền</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="39" t="inlineStr">
         <is>
           <t>Đã ghép</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J4" s="39" t="inlineStr">
         <is>
           <t>09:33
 "' ï
@@ -1659,50 +2594,50 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="39" t="inlineStr">
         <is>
           <t>z6042817618842_c41f77.jpg</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="40" t="n">
         <v>300000</v>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="39" t="inlineStr">
         <is>
           <t>DH1005 lan 1</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="39" t="inlineStr">
         <is>
           <t>HOANG THU HA</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="39" t="inlineStr">
         <is>
           <t>DT26101200871</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="39" t="inlineStr">
         <is>
           <t>12/10/2026 10:02:19</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="39" t="inlineStr">
         <is>
           <t>DH1005</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="39" t="inlineStr">
         <is>
           <t>có mã đơn, có tên khách</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I5" s="39" t="inlineStr">
         <is>
           <t>Đã ghép</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="J5" s="39" t="inlineStr">
         <is>
           <t>10:02
 aul
@@ -1722,50 +2657,50 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="39" t="inlineStr">
         <is>
           <t>z6042817733015_77ab02.jpg</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="40" t="n">
         <v>260000</v>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="39" t="inlineStr">
         <is>
           <t>DH1005 lan 2</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="39" t="inlineStr">
         <is>
           <t>HOANG THU HA</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="39" t="inlineStr">
         <is>
           <t>FT26285310927</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="39" t="inlineStr">
         <is>
           <t>12/10/2026 15:47:52</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="39" t="inlineStr">
         <is>
           <t>DH1005</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="39" t="inlineStr">
         <is>
           <t>có mã đơn, có tên khách</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="39" t="inlineStr">
         <is>
           <t>Đã ghép</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="J6" s="39" t="inlineStr">
         <is>
           <t>15:47 a l
 Sen Vàng Bank
@@ -1782,46 +2717,46 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="41" t="inlineStr">
         <is>
           <t>z6042817840331_e0d5b8.jpg</t>
         </is>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="42" t="n">
         <v>250000</v>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="41" t="inlineStr">
         <is>
           <t>chuyen tien</t>
         </is>
       </c>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="D7" s="41" t="n"/>
+      <c r="E7" s="41" t="inlineStr">
         <is>
           <t>FT26285322108</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="41" t="inlineStr">
         <is>
           <t>12/10/2026 10:50:31</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="41" t="inlineStr">
         <is>
           <t>DH1006</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="41" t="inlineStr">
         <is>
           <t>Chỉ đúng số tiền, chưa đủ để ghép</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="I7" s="41" t="inlineStr">
         <is>
           <t>Gợi ý, cần người xác nhận</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="J7" s="41" t="inlineStr">
         <is>
           <t>40:50 "Am l
 Biên Xanh Bank
@@ -1839,50 +2774,50 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="39" t="inlineStr">
         <is>
           <t>z6042817921456_19ce4d.jpg</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="40" t="n">
         <v>1500000</v>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="39" t="inlineStr">
         <is>
           <t>DO GIA HUY thanh toan</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="39" t="inlineStr">
         <is>
           <t>DO GIA HUY</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="39" t="inlineStr">
         <is>
           <t>DT26101201544</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="39" t="inlineStr">
         <is>
           <t>12/10/2026 11:05:44</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="39" t="inlineStr">
         <is>
           <t>DH1007</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" s="39" t="inlineStr">
         <is>
           <t>có tên khách, đúng số tiền</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I8" s="39" t="inlineStr">
         <is>
           <t>Đã ghép</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="J8" s="39" t="inlineStr">
         <is>
           <t>11:05
 aul
@@ -1902,38 +2837,42 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="39" t="inlineStr">
         <is>
           <t>z6042818034470_5d2a90.png</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="40" t="n">
         <v>5400000</v>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="39" t="inlineStr">
         <is>
           <t>DH1008 TT HD 00000126</t>
         </is>
       </c>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="D9" s="39" t="n"/>
+      <c r="E9" s="39" t="n"/>
+      <c r="F9" s="39" t="inlineStr">
+        <is>
+          <t>12/10/2026 11:31:02</t>
+        </is>
+      </c>
+      <c r="G9" s="39" t="inlineStr">
         <is>
           <t>DH1008</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H9" s="39" t="inlineStr">
         <is>
           <t>có mã đơn, có tên khách, đúng số tiền</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I9" s="39" t="inlineStr">
         <is>
           <t>Đã ghép</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="J9" s="39" t="inlineStr">
         <is>
           <t>Kết quả giao dịch: Chuyên khoản thành công
 1903 2222 1111
@@ -1957,38 +2896,38 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="39" t="inlineStr">
         <is>
           <t>z6042818115902_b8e6c3.jpg</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="40" t="n">
         <v>800000</v>
       </c>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="C10" s="39" t="n"/>
+      <c r="D10" s="39" t="n"/>
+      <c r="E10" s="39" t="n"/>
+      <c r="F10" s="39" t="inlineStr">
         <is>
           <t>11:42 - 12/10/2026</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="39" t="inlineStr">
         <is>
           <t>DH1009</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H10" s="39" t="inlineStr">
         <is>
           <t>có mã đơn, có tên khách</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="I10" s="39" t="inlineStr">
         <is>
           <t>Đã ghép</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="J10" s="39" t="inlineStr">
         <is>
           <t>11:42
 "' ï
@@ -2009,46 +2948,46 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="39" t="inlineStr">
         <is>
           <t>z6042818207719_0f4ad1.jpg</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
+      <c r="B11" s="40" t="n">
         <v>350000</v>
       </c>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="C11" s="39" t="n"/>
+      <c r="D11" s="39" t="inlineStr">
         <is>
           <t>DANG HUU PHUOC</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="39" t="inlineStr">
         <is>
           <t>FT26285512870</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" s="39" t="inlineStr">
         <is>
           <t>42/10/2026 13:22:16</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" s="39" t="inlineStr">
         <is>
           <t>DH1010</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H11" s="39" t="inlineStr">
         <is>
           <t>có mã đơn, có tên khách, đúng số tiền</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="I11" s="39" t="inlineStr">
         <is>
           <t>Đã ghép</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="J11" s="39" t="inlineStr">
         <is>
           <t>13:22 wt a)
 Sen Vang Bank
@@ -2065,48 +3004,48 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="43" t="inlineStr">
         <is>
           <t>z6042818350288_6ac2e5.jpg</t>
         </is>
       </c>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="B12" s="44" t="n"/>
+      <c r="C12" s="43" t="inlineStr">
         <is>
           <t>DH1011 Ngo Thi Kim</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="43" t="inlineStr">
         <is>
           <t>NGO THI KIM</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="43" t="inlineStr">
         <is>
           <t>DT26101202230</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F12" s="43" t="inlineStr">
         <is>
           <t>12/10/2026 14:01:33</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G12" s="43" t="inlineStr">
         <is>
           <t>DH1011</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H12" s="43" t="inlineStr">
         <is>
           <t>có mã đơn, có tên khách</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="I12" s="43" t="inlineStr">
         <is>
           <t>Không đọc được số tiền; mở ảnh kiểm tra</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="J12" s="43" t="inlineStr">
         <is>
           <t>Người chuyển: NGO THI KIM
 Từ tài khoản: 2201 8899 7766
@@ -2120,42 +3059,46 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="39" t="inlineStr">
         <is>
           <t>z6042818462531_2e7b9f.png</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="40" t="n">
         <v>3240000</v>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="39" t="inlineStr">
         <is>
           <t>DH1012 thanh toan hoa don 00000127</t>
         </is>
       </c>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="D13" s="39" t="n"/>
+      <c r="E13" s="39" t="inlineStr">
         <is>
           <t>FT26285618833</t>
         </is>
       </c>
-      <c r="F13" s="3" t="n"/>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="F13" s="39" t="inlineStr">
+        <is>
+          <t>12/40/2026 14:20:09</t>
+        </is>
+      </c>
+      <c r="G13" s="39" t="inlineStr">
         <is>
           <t>DH1012</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H13" s="39" t="inlineStr">
         <is>
           <t>có mã đơn, có tên khách, đúng số tiền</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="I13" s="39" t="inlineStr">
         <is>
           <t>Đã ghép</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr">
+      <c r="J13" s="39" t="inlineStr">
         <is>
           <t>Kết quả giao dịch: Chuyên khoản thành công
 1903 2222 1111
@@ -2179,46 +3122,46 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="39" t="inlineStr">
         <is>
           <t>z6042818573004_d9f310.jpg</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="40" t="n">
         <v>1550000</v>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="39" t="inlineStr">
         <is>
           <t>DH1013 DH1014</t>
         </is>
       </c>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="D14" s="39" t="n"/>
+      <c r="E14" s="39" t="inlineStr">
         <is>
           <t>FT26285702264</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F14" s="39" t="inlineStr">
         <is>
           <t>12/10/2026 14:48:55</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G14" s="39" t="inlineStr">
         <is>
           <t>DH1013, DH1014</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H14" s="39" t="inlineStr">
         <is>
           <t>1 lần chuyển cho 2 đơn: có mã các đơn, tổng tiền khớp</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="I14" s="39" t="inlineStr">
         <is>
           <t>Đã ghép, chia cho 2 đơn</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="J14" s="39" t="inlineStr">
         <is>
           <t>14:48 || o_o
 Bién Xanh Bank
@@ -2236,46 +3179,46 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="39" t="inlineStr">
         <is>
           <t>z6042818680147_41b8ac.jpg</t>
         </is>
       </c>
-      <c r="B15" s="8" t="n">
+      <c r="B15" s="40" t="n">
         <v>2100000</v>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="39" t="inlineStr">
         <is>
           <t>DH1015 Ly Thanh Tam</t>
         </is>
       </c>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="D15" s="39" t="n"/>
+      <c r="E15" s="39" t="inlineStr">
         <is>
           <t>MM2610121537</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F15" s="39" t="inlineStr">
         <is>
           <t>15:37 - 12/10/2026</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G15" s="39" t="inlineStr">
         <is>
           <t>DH1015</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H15" s="39" t="inlineStr">
         <is>
           <t>có mã đơn, có tên khách, đúng số tiền</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="I15" s="39" t="inlineStr">
         <is>
           <t>Đã ghép</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr">
+      <c r="J15" s="39" t="inlineStr">
         <is>
           <t>15:37
 "' ï
@@ -2296,46 +3239,46 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="41" t="inlineStr">
         <is>
           <t>z6042818791260_a3c6d2.jpg</t>
         </is>
       </c>
-      <c r="B16" s="11" t="n">
+      <c r="B16" s="42" t="n">
         <v>430000</v>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C16" s="41" t="inlineStr">
         <is>
           <t>DH0987 Phan Van Quang</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D16" s="41" t="inlineStr">
         <is>
           <t>PHAN VAN QUANG</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E16" s="41" t="inlineStr">
         <is>
           <t>FT26285800412</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F16" s="41" t="inlineStr">
         <is>
           <t>12/10/2026 16:12:40</t>
         </is>
       </c>
-      <c r="G16" s="6" t="n"/>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="G16" s="41" t="n"/>
+      <c r="H16" s="41" t="inlineStr">
         <is>
           <t>Không thấy mã đơn, SĐT, tên khách hay số tiền nào khớp</t>
         </is>
       </c>
-      <c r="I16" s="6" t="inlineStr">
+      <c r="I16" s="41" t="inlineStr">
         <is>
           <t>Chưa ghép được; xem ảnh và tìm đơn</t>
         </is>
       </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="J16" s="41" t="inlineStr">
         <is>
           <t>46:12 | MHỊ
 Sen Vàng Bank
@@ -2352,42 +3295,42 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="43" t="inlineStr">
         <is>
           <t>z6042819002388_3b9e01.jpg</t>
         </is>
       </c>
-      <c r="B17" s="10" t="n">
+      <c r="B17" s="44" t="n">
         <v>320000</v>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="43" t="inlineStr">
         <is>
           <t>0912345678 thanh toan</t>
         </is>
       </c>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="D17" s="43" t="n"/>
+      <c r="E17" s="43" t="inlineStr">
         <is>
           <t>MM2610120933</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" s="43" t="inlineStr">
         <is>
           <t>09:33 - 12/10/2026</t>
         </is>
       </c>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="G17" s="43" t="n"/>
+      <c r="H17" s="43" t="inlineStr">
         <is>
           <t>có số điện thoại, đúng số tiền</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="I17" s="43" t="inlineStr">
         <is>
           <t>Trùng với ảnh z6042817502117_3b9e01.jpg; không cộng tiền</t>
         </is>
       </c>
-      <c r="J17" s="5" t="inlineStr">
+      <c r="J17" s="43" t="inlineStr">
         <is>
           <t>09:33
 "' ï
@@ -2408,28 +3351,28 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="43" t="inlineStr">
         <is>
           <t>z6042819115630_7e21aa.jpg</t>
         </is>
       </c>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="inlineStr">
+      <c r="B18" s="44" t="n"/>
+      <c r="C18" s="43" t="n"/>
+      <c r="D18" s="43" t="n"/>
+      <c r="E18" s="43" t="n"/>
+      <c r="F18" s="43" t="n"/>
+      <c r="G18" s="43" t="n"/>
+      <c r="H18" s="43" t="inlineStr">
         <is>
           <t>Không thấy mã đơn, SĐT, tên khách hay số tiền nào khớp</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="I18" s="43" t="inlineStr">
         <is>
           <t>Không đọc được số tiền; có thể không phải biên nhận</t>
         </is>
       </c>
-      <c r="J18" s="5" t="inlineStr">
+      <c r="J18" s="43" t="inlineStr">
         <is>
           <t>Mau bó hoa số 3 —- còn hàng không shop?</t>
         </is>

</xml_diff>